<commit_message>
BSI.IT.27.C7: final package - samples and policies for period 07/2025-06/2026
- Add Sample of 1 for Sample 1 (2025 Q3); 2026 Q1 renamed as Sample 2
- Replace IAM Standard v11.0 (07/28/2026, after period) with v10.0 (09/29/2025, in effect)
- Update criteria references in WP2, walkthrough and samples; index refreshed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GtAt3iBzX5VYFEMTgXwPkP
</commit_message>
<xml_diff>
--- a/BSI.IT.27.C7 Network Device Admin Accoun/BSI.IT.27.C7 Final 07.2025-06.2026/00 Final Workpaper/BSI.IT.27.C7.05 Testing Walkthrough - Step by Step.xlsx
+++ b/BSI.IT.27.C7 Network Device Admin Accoun/BSI.IT.27.C7 Final 07.2025-06.2026/00 Final Workpaper/BSI.IT.27.C7.05 Testing Walkthrough - Step by Step.xlsx
@@ -588,7 +588,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Control statement; PAM Recertification Procedure v2.0 (04/22/2026) sec. 2 &amp; 8.1 C7; IAM Std v11.0 SUS.IAMS.4.2.5.6, 4.2.5.9, 4.2.5.19</t>
+          <t>Control statement; PAM Recertification Procedure v2.0 (04/22/2026) sec. 2 &amp; 8.1 C7; IAM Std v10.0 (09/29/2025) SUS.IAMS.4.2.5.6, 4.2.5.9, 4.2.5.19</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>IAM Standard (CUSO) v11.0 07.28.26 sec. 4.2.5; PAM Recertification Procedure (BSI) v2.0 04.22.26</t>
+          <t>IAM Standard v10.0 (approved 09/29/2025) sec. 4.2.5; PAM Recertification Procedure (BSI) v2.0 (approved 04/22/2026)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -19900,7 +19900,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>BSI.IT.27.C7.01.Identity and Access Management Standard (CUSO) 07.28.26.pdf</t>
+          <t>BSI.IT.27.C7.01 Identity and Access Management Standard v10.0 09.29.2025.pdf</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -19910,22 +19910,22 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Standard v11.0 (07/28/2026)</t>
+          <t>Standard v10.0 (approved 09/29/2025) - in effect in the period</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>777 KB</t>
+          <t>647 KB</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Criteria SUS.IAMS.4.2.5.x</t>
+          <t>Criteria SUS.IAMS.4.2.5.x (4.2.5.19 privileged access at least semi-annually; 4.2.5.21 revocation within 30 business days)</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>35484fd4951ac6439d9e4aee56437c38</t>
+          <t>bc6cbef4c58ffd183348884d02a16cee</t>
         </is>
       </c>
     </row>
@@ -19952,7 +19952,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Control C7, quarterly SOX recertification, revocation steps 9-10</t>
+          <t>Control C7, quarterly SOX recertification, revocation steps 9-10 (v1.0 of 04/22/2025 applied before 04/22/2026)</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -20079,7 +20079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -20452,41 +20452,76 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Criteria</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>IAM Standard v9.0 (in effect 07/01-09/28/2025) and PAM Recertification Procedure v1.0 (04/22/2025, in effect until 04/21/2026) - the versions in force at the 2025 Q3 review</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Policy administration</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Confirms criteria at the 2025 Q3 review date; v10.0 / v2.0 requirements used are unchanged in v11.0 (SUS.IAMS.4.2.5.x).</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Scope</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Decision whether Network_support (PAM Definition 3.2) is in scope</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>InfoSec / control owner</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>Scope observation.</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="11" t="inlineStr">
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>Essential to close the testing: #1 (2025 Q4) and #2 (management response). #3-#5 decide whether any exception can be cleared.</t>
         </is>
@@ -20494,8 +20529,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A16:G16"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A15:G15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
BSI.IT.27.C7: align final workpaper to the 9-step test procedure
- WP2 CPA test steps rewritten to the 9-step procedure; steps 6-7 result added
- Walkthrough tab 8_Procedure Coverage maps each step to work, evidence and result
- Evidence status: ServiceNow tickets / exception and escalation records requested

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GtAt3iBzX5VYFEMTgXwPkP
</commit_message>
<xml_diff>
--- a/BSI.IT.27.C7 Network Device Admin Accoun/BSI.IT.27.C7 Final 07.2025-06.2026/00 Final Workpaper/BSI.IT.27.C7.05 Testing Walkthrough - Step by Step.xlsx
+++ b/BSI.IT.27.C7 Network Device Admin Accoun/BSI.IT.27.C7 Final 07.2025-06.2026/00 Final Workpaper/BSI.IT.27.C7.05 Testing Walkthrough - Step by Step.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_Exceptions" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_Sources" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7_Evidence Status" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8_Procedure Coverage" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'4_Item Detail'!$A$3:$W$152</definedName>
@@ -20079,7 +20080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -20487,41 +20488,76 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Steps 6-7</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>ServiceNow revocation tickets for the 2025 Q3 / 2026 Q1 revocations and any exception / issue record (escalation, owner, due date, tracking to closure) for the A5 / A6 exceptions</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>PAM / IAM; control owner</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Needed to test exception handling and escalation (procedure steps 6-7); without it steps 6-7 remain Fail (not evidenced).</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Scope</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Decision whether Network_support (PAM Definition 3.2) is in scope</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>InfoSec / control owner</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>Scope observation.</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="11" t="inlineStr">
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>Essential to close the testing: #1 (2025 Q4) and #2 (management response). #3-#5 decide whether any exception can be cleared.</t>
         </is>
@@ -20529,8 +20565,342 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A16:G16"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A17:G17"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Coverage of the 9-step test procedure - period 07/01/2025 - 06/30/2026 - samples 2025 Q3 and 2026 Q1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Test procedure step</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Work performed and result</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Where documented</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="150" customHeight="1">
+      <c r="A4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Obtain Evidence</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Campaign documentation, certification records, reviewer decisions, account populations, revocation populations, campaign completion records, evidence of removals by PAM/IAM.</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Obtained: 2025 Q3 and 2026 Q1 SailPoint Manager / Owner certification exports (decisions, decision maker, sign-off dates), AD extracts 11/25/2025 and 05/15/2026, Netwrix removal logs, IAM Standard v10.0, PAM Recertification Procedure v2.0, PAM Definition of Privilege v10.0. Not provided: 2025 Q4 certification, ServiceNow revocation tickets, 2026 Q1 campaign completion screenshot.</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Tabs 6, 7; 02 Evidence; 01 Policies</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Pass (observation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="150" customHeight="1">
+      <c r="A5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Validate Report Completeness and Accuracy</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Reconcile the certified population to the authoritative source; investigate discrepancies.</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Certified memberships reconciled to the BSI AD extracts (authoritative source). 2025 Q3: differences explained (revoked and removed; N584407 left after review; X842395, MIA25172 / MIA25175 ISEAdmin added after launch and certified in 2026 Q1). 2026 Q1: 58/58 AD members certified; 3 extra = revoked and removed. Report observations: Q1 export rows repeated 5x (de-duplicated), IAMS termination vs AD expiration inconsistent.</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Step 8; Sample of 1 Exhibit C1; tab 4</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Pass (observation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="150" customHeight="1">
+      <c r="A6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Validate Population and Scope</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>All in-scope administrator, user and service accounts included; none excluded.</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Scope = 4 privileged network AD groups (PAM Definition of Privilege sec. 3.3). 88 memberships in 2025 Q3 and 61 in 2026 Q1, person and service accounts, 100% tested; no in-scope account excluded. Observation: Network_support (sec. 3.2) not in scope - management to confirm.</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Steps 1, 7; tab 3</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>Pass (observation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="150" customHeight="1">
+      <c r="A7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Verify Control Execution</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Sample per RCSA methodology incl. revocations; InfoSec initiated the campaign; authorized manager / owner; decisions documented and completed; revocations identified through the review.</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Sample: 2 quarterly campaigns (medium assurance), 100% of memberships including all 36 revocation decisions. Initiation: campaigns launched in SailPoint by the PAM / IAM team (8/1 and 8/4/2025; 4/9/2026) per Procedure sec. 8 steps 1-7. Reviewer: line managers / owners, no self-review. Decisions: 88/88 and 61/61 with sign-off. Revocations identified: 33 in 2025 Q3, 3 in 2026 Q1. BUT the reviewers approved access that should have been revoked (A5: 2025 Q3 14, 2026 Q1 30 memberships).</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Steps 6, 9-12; tab 3; tab 5</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Fail (A5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="150" customHeight="1">
+      <c r="A8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Validate Control Results</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Revoked access removed by PAM/IAM within SLA after the review and consistent with the decision.</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>2025 Q3: 33 revoked 8/28/2025, removed 9/2-9/8/2025 (Netwrix) - within 30 business days and matching the decisions; 6 memberships (X453396 x2, MIA25142 x2, MIA25172, MIA25175) were members again on 11/25/2025 - removal not sustained. 2026 Q1: N596764 x2 removed 4/24/2026, MIAYPER 4/17/2026 - within SLA, absent from AD 05/15/2026.</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Step 13; Sample of 1 Exhibits B4 / B5</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Fail (A6 - 2025 Q3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="150" customHeight="1">
+      <c r="A9" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Verify Exception Handling</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Where revocations were late, reviews incomplete or reviewer authorization missing, verify the exception was documented and managed per procedure.</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>No reviews were incomplete and no reviewer authorization issues were found. The exceptions found by testing (approved terminated / disabled accounts; 6 revoked memberships present again in AD) were not identified, documented or managed by the PAM / IAM team - no exception record, ticket or comment exists in the evidence (the 2025 Q3 AD extract shows the revoked members without comment).</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Tab 5; Evidence Status #2, #12</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Fail (not evidenced)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="150" customHeight="1">
+      <c r="A10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Verify Escalation and Remediation</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Exceptions escalated; remediation documented, assigned and tracked to resolution.</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>No escalation, remediation plan, owner or tracking was provided for the exceptions; the same accounts were approved again in the next review (2025 Q3 -&gt; 2026 Q1), showing they were not remediated within the period. Management response and issue / action driver required.</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Tab 5; Evidence Status #2, #12</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Fail (not evidenced)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="150" customHeight="1">
+      <c r="A11" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Assess Risk Mitigation</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Does the review identify inappropriate access and drive timely revocation?</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Partially. The review is initiated, complete and performed by the right reviewers, and revocations that were raised were removed on time. However it did not identify terminated / disabled accounts in Cisco Network Administrators and ISEAdmin in either review, and removals were not sustained, so the risk of inappropriate privileged network access is not fully mitigated.</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Tab 3 conclusion; WP2 CPA</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Fail - Needs Improvement</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="150" customHeight="1">
+      <c r="A12" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Summarize Testing Coverage</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Coverage of completeness / accuracy, scope, initiation, reviewer authorization, execution, revocation decisions, timeliness, exception management, escalation, risk mitigation.</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Completeness &amp; accuracy: Pass (obs.). Scope: Pass (obs.). Initiation / frequency: Pass (obs. - 2025 Q4 missing). Reviewer authorization: Pass. Certification execution: Pass. Revocation decisions / appropriateness: Fail. Timeliness of removal: Pass within SLA, Fail on persistence (2025 Q3). Exception management: Fail (not evidenced). Escalation: Fail (not evidenced). Risk mitigation: Fail. Overall: 2 of 2 samples Fail - Needs Improvement.</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>This tab; WP2 C39</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Fail - Needs Improvement</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>